<commit_message>
Remove '全域' from storm surge building collapse layer name
Change the layer from a subcategory with '全域' child to a direct
menu item named '家屋倒壊等氾濫想定区域（氾濫流・高潮）'.
</commit_message>
<xml_diff>
--- a/メニュー/メニュー.xlsx
+++ b/メニュー/メニュー.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z1009"/>
+  <dimension ref="A1:M229"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2039,11 +2039,8 @@
       <c r="A97" t="str">
         <v>防災</v>
       </c>
-      <c r="B97" t="str">
+      <c r="C97" t="str">
         <v>家屋倒壊等氾濫想定区域（氾濫流・高潮）</v>
-      </c>
-      <c r="C97" t="str">
-        <v>全域</v>
       </c>
       <c r="D97" t="str">
         <v>https://yaizu-smartcity.jp/tiles/yaizu-kaoku-tokai-hanranryu/tiles.json</v>
@@ -4343,7 +4340,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z1009"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M229"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>